<commit_message>
MAJ des entrées CDA (#122)
* MAJ-card-attributs-code

* update entrées CDA 297b5adb0c485659eb8ec7e94a48f9ff12d8e171
</commit_message>
<xml_diff>
--- a/fusionEntreesCDA/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
+++ b/fusionEntreesCDA/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-20T06:44:24+00:00</t>
+    <t>2026-04-20T07:29:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -4700,7 +4700,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" hidden="true">
+    <row r="33">
       <c r="A33" t="s" s="2">
         <v>167</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>75</v>
       </c>
       <c r="H33" t="s" s="2">
-        <v>74</v>
+        <v>160</v>
       </c>
       <c r="I33" t="s" s="2">
         <v>74</v>
@@ -5104,7 +5104,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="37" hidden="true">
+    <row r="37">
       <c r="A37" t="s" s="2">
         <v>176</v>
       </c>
@@ -5119,13 +5119,13 @@
         <v>62</v>
       </c>
       <c r="F37" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G37" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H37" t="s" s="2">
-        <v>74</v>
+        <v>160</v>
       </c>
       <c r="I37" t="s" s="2">
         <v>74</v>
@@ -5207,7 +5207,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>180</v>
       </c>
@@ -5222,13 +5222,13 @@
         <v>181</v>
       </c>
       <c r="F38" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>74</v>
+        <v>160</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>74</v>
@@ -5516,7 +5516,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" hidden="true">
+    <row r="41">
       <c r="A41" t="s" s="2">
         <v>194</v>
       </c>
@@ -5531,13 +5531,13 @@
         <v>195</v>
       </c>
       <c r="F41" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G41" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>74</v>
+        <v>160</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>74</v>

</xml_diff>

<commit_message>
Mise à jour cardinalité (#125) 3e1f2de51fef0803f685bb629d106e92500326a5
</commit_message>
<xml_diff>
--- a/fusionEntreesCDA/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
+++ b/fusionEntreesCDA/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-20T07:29:37+00:00</t>
+    <t>2026-04-20T13:53:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -5531,7 +5531,7 @@
         <v>195</v>
       </c>
       <c r="F41" t="s" s="2">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G41" t="s" s="2">
         <v>75</v>

</xml_diff>